<commit_message>
feat: nuevos patrones de deteccion de cuadros en resumenes
Agrega deteccion de frases 'cuyo detalle... siguiente cuadro:' y 'se describen en el siguiente cuadro:' para cortar tablas correctamente en los articulos extraidos de los PDFs.
</commit_message>
<xml_diff>
--- a/data/resoluciones_pendientes.xlsx
+++ b/data/resoluciones_pendientes.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pendientes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="pendientes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -140,8 +140,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResolucionesPendientes" displayName="ResolucionesPendientes" ref="A1:R2" headerRowCount="1">
-  <autoFilter ref="A1:R2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResolucionesPendientes" displayName="ResolucionesPendientes" ref="A1:R9" headerRowCount="1">
+  <autoFilter ref="A1:R9"/>
   <tableColumns count="18">
     <tableColumn id="1" name="archivo_pdf"/>
     <tableColumn id="2" name="ruta_pdf"/>
@@ -455,13 +455,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="82" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
@@ -573,12 +573,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>64-RD-0156-2026-04.pdf</t>
+          <t>64-RD-0160-2026-06.pdf</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>D:\Archivos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0156-2026-04.pdf</t>
+          <t>D:\Archivos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0160-2026-06.pdf</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -608,12 +608,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>0156-2026-ANA-AAA.MDD</t>
+          <t>0160-2026-ANA-AAA.MDD</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -623,7 +623,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>26/05/2026</t>
+          <t>28/05/2026</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -633,30 +633,674 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>RD N° 0156-2026-ANA-AAA.MDD</t>
+          <t>RD N° 0160-2026-ANA-AAA.MDD</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>ARTÍCULO 1.- OTORGAR Autorización de uso temporal de un área de terreno de la bifurcación izquierda del rio Inambari para siembra de cultivos de 5.00 ha a favor del señor DINER SANCHEZ MOLINA, identificado con DNI N° 71515428, dicha área se ubica en el sector Ponal, distrito de Inambari, provincia de Tambopata y departamento de Madre de Dios;</t>
+          <t>ARTÍCULO 1.- DECLARAR la EXTINCIÓN de Licencia de uso de agua subterránea en vía de regularización con fines mineros, otorgada mediante la Resolución Administrativa N° 452- 2012-ANA-ALAM de fecha 14.11.2012, a favor del señor Víctor Damaso Araos Fuentes, identificado con DNI N° 04813153 y RUC N° 10048131536, por la causal prevista en el numeral 1 del artículo 71 de la Ley de Recursos Hídricos: Muerte del titular del derecho.</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>ARTÍCULO 1.- OTORGAR Autorización de uso temporal de un área de terreno de la bifurcación izquierda del rio Inambari para siembra de cultivos de 5.00 ha a favor del señor DINER SANCHEZ MOLINA, identificado con DNI N° 71515428, dicha área se ubica en el sector Ponal, distrito de Inambari, provincia de Tambopata y departamento de Madre de Dios;</t>
+          <t>ARTÍCULO 1.- DECLARAR la EXTINCIÓN de Licencia de uso de agua subterránea en vía de regularización con fines mineros, otorgada mediante la Resolución Administrativa N° 452- 2012-ANA-ALAM de fecha 14.11.2012, a favor del señor Víctor Damaso Araos Fuentes, identificado con DNI N° 04813153 y RUC N° 10048131536, por la causal prevista en el numeral 1 del artículo 71 de la Ley de Recursos Hídricos: Muerte del titular del derecho.</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>ARTÍCULO 2.- PRECISAR que la presente autorización tiene un plazo de vigencia de cinco (05) años, la misma que se computará a partir de la emisión de la presente resolución.</t>
+          <t>ARTÍCULO 2.- REVERTIR al dominio del Estado, el volumen anual de 26 956.80 m³, como consecuencia de la declaratoria de extinción de la licencia de uso de agua, proveniente de la fuente de agua subterránea.</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>ARTÍCULO 3.- REGISTRAR la presente autorización en el inventario de áreas ocupadas de las fajas marginales de fuentes naturales de agua, en cumplimiento de lo establecido en el artículo 5 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales.</t>
+          <t>ARTÍCULO 3.- INSCRIBIR el presente acto administrativo en el Registro Administrativo de Derechos de Uso de Agua (RADA).</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>59-RD-0161-2026-04.pdf</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>D:\Archivos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0161-2026-04.pdf</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>ALA Tahuamanu Madre de Dios</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>AAA Madre de Dios</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Resoluciones Emitidas por el ANA</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>De las Autoridades Administrativas del Agua</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>0161-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>161</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>28/05/2026</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00 am</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>RD N° 0161-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- OTORGAR, Autorización de Uso de Agua subterránea para la ejecución de obras para el proyecto denominado “Mejoramiento y ampliación del servicio educación inicial en las instituciones educativas Nro 292 San Bernardo, Nro 312 Tres Islas, Nro 313 Palma Real, Nro 378 los Pihuichitos Santa Teresita, Nro 398 el castañal y Nro 395 Primero de Agosto del Distrito de Tambopata, provincia de Tambopata - Madre de Dios”, a favor del GOBIERNO REGIONAL MADRE DE DIOS con RUC N° 2057143200, cuyo aprovechamiento de agua será por un volumen anual de hasta 21 039.00 m 3.</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- OTORGAR, Autorización de Uso de Agua subterránea para la ejecución de obras para el proyecto denominado “Mejoramiento y ampliación del servicio educación inicial en las instituciones educativas Nro 292 San Bernardo, Nro 312 Tres Islas, Nro 313 Palma Real, Nro 378 los Pihuichitos Santa Teresita, Nro 398 el castañal y Nro 395 Primero de Agosto del Distrito de Tambopata, provincia de Tambopata - Madre de Dios”, a favor del GOBIERNO REGIONAL MADRE DE DIOS con RUC N° 2057143200, cuyo aprovechamiento de agua será por un volumen anual de hasta 21 039.00 m 3.</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 2.- PRECISAR que la presente resolución tendrá un plazo de vigencia de uno (1) año que se computará a partir del día siguiente de la notificación de la presente resolución.</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 3.- INSCRIBIR el presente acto administrativo en el Registro Administrativo de Derechos de Uso de Agua (RADA).</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>64-RD-0162-2026-06.pdf</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>D:\Archivos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0162-2026-06.pdf</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>ALA Tambopata - Inambari</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>AAA Madre de Dios</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Resoluciones Emitidas por el ANA</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>De las Autoridades Administrativas del Agua</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>0162-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>162</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>28/05/2026</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00 am</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>RD N° 0162-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- DECLARAR la EXTINCIÓN de Licencia de uso de agua superficial con fines mineros, otorgada mediante la Resolución Administrativa N° 238-2010-ANA-ALAM de fecha 02.11.2010, a favor del señor Luis Ramos Valdez, identificado con DNI N° 04804738, por la causal prevista en el numeral 1 del artículo 71 de la Ley de Recursos Hídricos: Muerte del titular del derecho.</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- DECLARAR la EXTINCIÓN de Licencia de uso de agua superficial con fines mineros, otorgada mediante la Resolución Administrativa N° 238-2010-ANA-ALAM de fecha 02.11.2010, a favor del señor Luis Ramos Valdez, identificado con DNI N° 04804738, por la causal prevista en el numeral 1 del artículo 71 de la Ley de Recursos Hídricos: Muerte del titular del derecho.</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 2.- REVERTIR al dominio del Estado, el volumen anual de 22 755.60 m³, como consecuencia de la declaratoria de extinción de la licencia de uso de agua, proveniente de la fuente de agua superficial.</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 3.- INSCRIBIR el presente acto administrativo en el Registro Administrativo de Derechos de Uso de Agua (RADA).</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>64-RD-0163-2026-04.pdf</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>D:\Archivos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0163-2026-04.pdf</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ALA Tambopata - Inambari</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>AAA Madre de Dios</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Resoluciones Emitidas por el ANA</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>De las Autoridades Administrativas del Agua</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>0163-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>163</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00 am</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>RD N° 0163-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- APROBAR los estudios de huella máxima que conforma el “Estudio de delimitación de la faja marginal en un tramo de 550 metros en ambas márgenes de la quebrada Quintana, ubicado en el centro poblado Nueva, distrito de Huepetuhe, provincia de Manu, departamento de Madre de Dios”, elaborado por el Área Técnica de esta Autoridad Administrativa del Agua, conforme a la metodología establecida en artículo 10 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales.</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- APROBAR los estudios de huella máxima que conforma el “Estudio de delimitación de la faja marginal en un tramo de 550 metros en ambas márgenes de la quebrada Quintana, ubicado en el centro poblado Nueva, distrito de Huepetuhe, provincia de Manu, departamento de Madre de Dios”, elaborado por el Área Técnica de esta Autoridad Administrativa del Agua, conforme a la metodología establecida en artículo 10 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales.</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 2.- APROBAR a solicitud de parte, el ancho de la faja marginal de la quebrada Quintana en un tramo de 550 metros, un ancho mínimo de 9.00 metros y un máximo de 26.00 metros en la margen derecha y un ancho mínimo de 4.00 metros y un máximo de 32.00 metros en la margen izquierda, conforme a los alcances señalados en el artículo 4 y los criterios establecidos en el artículo 12 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales.</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 3.- APROBAR la delimitación de la faja marginal en el tramo materia de estudio de la quebrada Quintana, ubicada en el centro poblado Nueva, distrito de Huepetuhe, provincia de Manu, departamentos de Madre de Dios, de conformidad a la metodología establecida en el artículo 6 y el procedimiento establecido en el artículo 18 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales, cuyo detalle se encuentra dispuesto en el anexo y el plano que forman parte de la presente resolución.</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>64-RD-0164-2026-04.pdf</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>D:\Archivos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0164-2026-04.pdf</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ALA Tambopata - Inambari</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>AAA Madre de Dios</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Resoluciones Emitidas por el ANA</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>De las Autoridades Administrativas del Agua</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>0164-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>164</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00 am</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>RD N° 0164-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- APROBAR los estudios de huella máxima que conforma el Estudio de delimitación de la faja marginal en un tramo de 860 metros en ambas márgenes de la quebrada Seca, ubicado en el centro poblado Nueva, distrito de Huepetuhe, provincia de Manu, departamento de Madre de Dios”, elaborado por el área técnica de esta Autoridad Administrativa del Agua, conforme a la metodología establecida en artículo 10 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales.</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- APROBAR los estudios de huella máxima que conforma el Estudio de delimitación de la faja marginal en un tramo de 860 metros en ambas márgenes de la quebrada Seca, ubicado en el centro poblado Nueva, distrito de Huepetuhe, provincia de Manu, departamento de Madre de Dios”, elaborado por el área técnica de esta Autoridad Administrativa del Agua, conforme a la metodología establecida en artículo 10 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales.</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 2.- APROBAR a solicitud de parte, el ancho de la faja marginal de la quebrada Seca en un tramo de 860 m, un ancho mínimo de 4.00 m y un máximo de 71.00 m en la margen derecha y un ancho mínimo de 4.00 m y un máximo de 29.00 m en la margen izquierda, conforme a los alcances señalados en el artículo 4 y los criterios establecidos en el artículo 12 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales.</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 3.- APROBAR la delimitación de la faja marginal en el tramo materia de estudio de la quebrada Seca, ubicada en el centro poblado Nueva, distrito de Huepetuhe, provincia de Manu, departamentos de Madre de Dios, de conformidad a la metodología establecida en el artículo 6 y el procedimiento establecido en el artículo 18 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales, cuyo detalle se encuentra dispuesto en el anexo y el plano que forman parte de la presente resolución.</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>59-RD-0165-2026-08.pdf</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>D:\Archivos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0165-2026-08.pdf</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>ALA Tahuamanu Madre de Dios</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>AAA Madre de Dios</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Resoluciones Emitidas por el ANA</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>De las Autoridades Administrativas del Agua</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>0165-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>04/06/2026</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00 am</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>RD N° 0165-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- SANCIONAR a la UNIDAD EJECUTORA 1392 - SUB REGION MANU con RUC N° 20490448951, con una sanción administrativa de MULTA, equivalente a cero coma cincuenta (0,50) UIT, por la infracción calificada como leve en materia de agua, por la construcción de una estructura de captación conformada por una bocatoma ubicada en la quebrada Isla de Los Valles, con un ancho de 3.00 m, muro de encauzamiento de 1.50 m y barraje de 1.20 m, además de una cámara de captación de concreto con tapas metálicas y tubería de conducción de PVC de 3”, sin autorización de la Autoridad Nacional del Agua, cuyo detalle de infracción, sanción y fuente natural de agua se describen en el siguiente cuadro: PLAZOS INFRACTOR RUC RAZÓN SOCIAL CALIFICACIÓN TIPO MONTO (UIT) Multa Medida complem entaria 20490448951 UNIDAD EJECUTORA 1392 SUB REGIÓN MANU SANCIÓN Leve Multa 0.50 15 días hábiles 90 días DESCRIPCIÓN DE LOS HECHOS ORIGEN TIPO UNIDAD HIDROGRÁFICA Superficial Quebrada Intercuenca Alto Madre de Dios (46649) Construcción de una estructura de captación conformada por una bocatoma ubicada en la quebrada Isla de Los Valles, con un ancho de 3.00 m, muro de encauzamiento de 1.50 m y barraje de 1.20 m, además de una cámara de captación de concreto con tapas metálicas y tubería de conducción de PVC de 3”, sin contar con la autorización de ejecución de obras con fines de aprovechamiento hídrico correspondiente. UBICACIÓN GEOGRAFICA DE LA INFRACCIÓN.</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- SANCIONAR a la UNIDAD EJECUTORA 1392 - SUB REGION MANU con RUC N° 20490448951, con una sanción administrativa de MULTA, equivalente a cero coma cincuenta (0,50) UIT, por la infracción calificada como leve en materia de agua, por la construcción de una estructura de captación conformada por una bocatoma ubicada en la quebrada Isla de Los Valles, con un ancho de 3.00 m, muro de encauzamiento de 1.50 m y barraje de 1.20 m, además de una cámara de captación de concreto con tapas metálicas y tubería de conducción de PVC de 3”, sin autorización de la Autoridad Nacional del Agua, cuyo detalle de infracción, sanción y fuente natural de agua se describen en el siguiente cuadro: PLAZOS INFRACTOR RUC RAZÓN SOCIAL CALIFICACIÓN TIPO MONTO (UIT) Multa Medida complem entaria 20490448951 UNIDAD EJECUTORA 1392 SUB REGIÓN MANU SANCIÓN Leve Multa 0.50 15 días hábiles 90 días DESCRIPCIÓN DE LOS HECHOS ORIGEN TIPO UNIDAD HIDROGRÁFICA Superficial Quebrada Intercuenca Alto Madre de Dios (46649) Construcción de una estructura de captación conformada por una bocatoma ubicada en la quebrada Isla de Los Valles, con un ancho de 3.00 m, muro de encauzamiento de 1.50 m y barraje de 1.20 m, además de una cámara de captación de concreto con tapas metálicas y tubería de conducción de PVC de 3”, sin contar con la autorización de ejecución de obras con fines de aprovechamiento hídrico correspondiente. UBICACIÓN GEOGRAFICA DE LA INFRACCIÓN.</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 2.- DISPONER que el depósito de la multa impuesta sea pagada mediante depósito en las agencias del Banco de la Nación en la Cuenta Corriente N° 0000-877174 de la Autoridad Nacional del Agua (concepto multas por infracción) en el plazo de quince (15) días hábiles de notificado la presente resolución, bajo apercibimiento de iniciarse ejecución coactiva en caso de incumplimiento, debiendo alcanzar una copia del Boucher de depósito a la Administración Local de Agua Tahuamanu-Madre de Dios dentro del tercer día de efectuado el mismo.</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 3.- DISPONER como Medida Complementaria la suspensión de las obras en los cuerpos de agua y los bienes asociados a esta, que no hayan sido autorizados por la Autoridad Nacional del Agua, otorgándole a la imputada un plazo máximo de hasta noventa (90) días, a partir del día siguiente de la notificación de la presente resolución para que realice los trámites para la obtención de la Autorización de Ejecución de Obras de Alumbramiento de Agua Subterránea para la Obtención de la Licencia de Uso de Agua Subterránea, transcurrido el plazo señalado y en caso no cuente con la autorización correspondiente, se procederá con el sellado del pozo.</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>59-RD-0166-2026-04.pdf</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>D:\Archivos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0166-2026-04.pdf</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>ALA Tahuamanu Madre de Dios</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>AAA Madre de Dios</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Resoluciones Emitidas por el ANA</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>De las Autoridades Administrativas del Agua</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>0166-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>166</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>04/06/2026</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00 am</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>RD N° 0166-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- SANCIONAR al señor JORGE DAVID TRIGOSO REATEGUI identificado con DNI N° 04824031, con una AMONESTACIÓN ESCRITA, por la infracción calificada como leve en materia de agua, por utilizar el agua con fines de uso doméstico-poblacional, en el distrito Las Piedras, provincia de Tambopata, departamento de Madre de Dios, cuyo detalle de infracción, sanción y fuente natural de agua se describen en el siguiente cuadro: INFRACTOR DNI N° NOMBRE CALIFICACIÓN TIPO MONTO (UIT) PLAZO CUMPLIMIENTO (Días Hábiles) 04824031 JORGE DAVID TRIGOSO REATEGUI SANCIÓN LEVE Amonestación Escrito --- --- DESCRIPCIÓN DE LOS HECHOS CLASE TIPO NOMBRE UNIDAD HIDROGRÁFICA Utilizar el agua con fines de uso doméstico-poblacional sin el correspondiente derecho de uso otorgado por la Autoridad Nacional del Agua, en el distrito Las Piedras, provincia de Tambopata, departamento de Madre de Dios. Subterránea Pozo Mixto S/N Cuenca Orthon (4662) TIPIFICACIÓN COORDENADAS DEL POZO PERFORADO Art. 120 LEY RECURSOS HÍDRICOS Art. 277 REGLAMENTO LRH DÁTUM ZONA ESTE (m) NORTE (m) UTM WGS84 19 S 487 114 8 672 252 UBICACIÓN POLÍTICA DEPARTAMENTO PROVINCIA DISTRITO INFRACCIÓN 1. Utilizar el agua sin el correspondiente derecho de uso a. Usar, represar o desviar las aguas sin el correspondiente derecho de uso de agua o autorización de la Autoridad Nacional del Agua FUENTE NATURAL DE AGUA Madre de Dios Tambopata Las Piedras.</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- SANCIONAR al señor JORGE DAVID TRIGOSO REATEGUI identificado con DNI N° 04824031, con una AMONESTACIÓN ESCRITA, por la infracción calificada como leve en materia de agua, por utilizar el agua con fines de uso doméstico-poblacional, en el distrito Las Piedras, provincia de Tambopata, departamento de Madre de Dios, cuyo detalle de infracción, sanción y fuente natural de agua se describen en el siguiente cuadro: INFRACTOR DNI N° NOMBRE CALIFICACIÓN TIPO MONTO (UIT) PLAZO CUMPLIMIENTO (Días Hábiles) 04824031 JORGE DAVID TRIGOSO REATEGUI SANCIÓN LEVE Amonestación Escrito --- --- DESCRIPCIÓN DE LOS HECHOS CLASE TIPO NOMBRE UNIDAD HIDROGRÁFICA Utilizar el agua con fines de uso doméstico-poblacional sin el correspondiente derecho de uso otorgado por la Autoridad Nacional del Agua, en el distrito Las Piedras, provincia de Tambopata, departamento de Madre de Dios. Subterránea Pozo Mixto S/N Cuenca Orthon (4662) TIPIFICACIÓN COORDENADAS DEL POZO PERFORADO Art. 120 LEY RECURSOS HÍDRICOS Art. 277 REGLAMENTO LRH DÁTUM ZONA ESTE (m) NORTE (m) UTM WGS84 19 S 487 114 8 672 252 UBICACIÓN POLÍTICA DEPARTAMENTO PROVINCIA DISTRITO INFRACCIÓN 1. Utilizar el agua sin el correspondiente derecho de uso a. Usar, represar o desviar las aguas sin el correspondiente derecho de uso de agua o autorización de la Autoridad Nacional del Agua FUENTE NATURAL DE AGUA Madre de Dios Tambopata Las Piedras.</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 2.- DISPONER como Medida Complementaria el cese de la utilización ilegítima del recurso hídrico, efectuado por el señor Jorge David Trigoso Reategui, otorgándole un plazo máximo de hasta tres (03) meses, computados a partir del día siguiente de la notificación de la presente resolución, para que regularice y obtenga el derecho de uso de agua correspondiente.</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 3.- DISPONER que la Administración Local de Agua Tahuamanu-Madre de Dios, verifique el cumplimiento de lo dispuesto en la Medida Complementaria.</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>59-RD-0167-2026-05.pdf</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>D:\Archivos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0167-2026-05.pdf</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>ALA Tahuamanu Madre de Dios</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>AAA Madre de Dios</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Resoluciones Emitidas por el ANA</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>De las Autoridades Administrativas del Agua</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>0167-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>167</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>04/06/2026</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00 am</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>RD N° 0167-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- SANCIONAR a la señora EUSEBIA JULIANA COLQUE FLORES, identificada con DNI N° 04827841, con una AMONESTACIÓN ESCRITA, por la infracción calificada como leve en materia de agua, por utilizar el agua con fines de uso doméstico-poblacional en el sector Santa Rosa - Km 504, Carretera Interoceánica Puerto Maldonado - Iñapari, distrito de Las Piedras, provincia de Tambopata, departamento de Madre de Dios, cuyo detalle de infracción, sanción y fuente natural de agua se describen en el siguiente cuadro: INFRACTOR DNI N° NOMBRE CALIFICACIÓN TIPO MONTO (UIT) PLAZO CUMPLIMIENTO (Días Hábiles) 04827841 EUSEBIA JULIANA COLQUE FLORES SANCIÓN LEVE Amonestación Escrita --- --- DESCRIPCIÓN DE LOS HECHOS ORIGEN NOMBRE LA FUENTE TIPO UNIDAD HIDROGRÁFICA Utilizar el agua con fines de uso doméstico-poblacional sin el correspondiente derecho de uso otorgado por la Autoridad Nacional del Agua, en el sector Santa Rosa - Km 504, Carretera Interoceánica Puerto Maldonado - Iñapari, distrito de Las Piedras, provincia de Tambopata, departamento de Madre de Dios. Subterránea Acuífero Cuenca Orthon (4662) Pozo Mixto Cuenca Orthon (4662) TIPIFICACIÓN COORDENADAS DEL POZO PERFORADO Art. 120 LEY RECURSOS HÍDRICOS Art. 277 REGLAMENTO LRH DÁTUM ZONA ESTE (m) NORTE (m) UTM WGS84 19 S 484 976 8 673 214 UBICACIÓN POLÍTICA DEPARTAMENTO PROVINCIA DISTRITO SECTOR INFRACCIÓN 1. Utilizar el agua sin el correspondiente derecho de uso a. Usar, represar o desviar las aguas sin el correspondiente derecho de uso de agua o autorización de la Autoridad Nacional del Agua FUENTE NATURAL DE AGUA Madre de Dios Tambopata Las Piedras Santa Rosa - Km 504, Carretera Interoceánica Puerto Maldonado - Iñapari.</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- SANCIONAR a la señora EUSEBIA JULIANA COLQUE FLORES, identificada con DNI N° 04827841, con una AMONESTACIÓN ESCRITA, por la infracción calificada como leve en materia de agua, por utilizar el agua con fines de uso doméstico-poblacional en el sector Santa Rosa - Km 504, Carretera Interoceánica Puerto Maldonado - Iñapari, distrito de Las Piedras, provincia de Tambopata, departamento de Madre de Dios, cuyo detalle de infracción, sanción y fuente natural de agua se describen en el siguiente cuadro: INFRACTOR DNI N° NOMBRE CALIFICACIÓN TIPO MONTO (UIT) PLAZO CUMPLIMIENTO (Días Hábiles) 04827841 EUSEBIA JULIANA COLQUE FLORES SANCIÓN LEVE Amonestación Escrita --- --- DESCRIPCIÓN DE LOS HECHOS ORIGEN NOMBRE LA FUENTE TIPO UNIDAD HIDROGRÁFICA Utilizar el agua con fines de uso doméstico-poblacional sin el correspondiente derecho de uso otorgado por la Autoridad Nacional del Agua, en el sector Santa Rosa - Km 504, Carretera Interoceánica Puerto Maldonado - Iñapari, distrito de Las Piedras, provincia de Tambopata, departamento de Madre de Dios. Subterránea Acuífero Cuenca Orthon (4662) Pozo Mixto Cuenca Orthon (4662) TIPIFICACIÓN COORDENADAS DEL POZO PERFORADO Art. 120 LEY RECURSOS HÍDRICOS Art. 277 REGLAMENTO LRH DÁTUM ZONA ESTE (m) NORTE (m) UTM WGS84 19 S 484 976 8 673 214 UBICACIÓN POLÍTICA DEPARTAMENTO PROVINCIA DISTRITO SECTOR INFRACCIÓN 1. Utilizar el agua sin el correspondiente derecho de uso a. Usar, represar o desviar las aguas sin el correspondiente derecho de uso de agua o autorización de la Autoridad Nacional del Agua FUENTE NATURAL DE AGUA Madre de Dios Tambopata Las Piedras Santa Rosa - Km 504, Carretera Interoceánica Puerto Maldonado - Iñapari.</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 2.- INSCRIBIR en el Registro de Sanciones, la sanción impuesta en el artículo 1 de la presente resolución, una vez que quede consentida o agote la vía administrativa.</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 3.- NOTIFICAR la presente resolución a la señora Eusebia Juliana Colque Flores en su domicilio; poner de conocimiento a la Administración Local de Agua Tahuamanu-Madre de Dios; y disponer su publicación en el portal web institucional de la Autoridad Nacional del Agua: www.ana.gob.pe.</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>

</xml_diff>

<commit_message>
chore: actualizar datos de carga - lote RDs 0181-0187 (7 publicadas)
</commit_message>
<xml_diff>
--- a/data/resoluciones_pendientes.xlsx
+++ b/data/resoluciones_pendientes.xlsx
@@ -140,8 +140,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResolucionesPendientes" displayName="ResolucionesPendientes" ref="A1:R3" headerRowCount="1">
-  <autoFilter ref="A1:R3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResolucionesPendientes" displayName="ResolucionesPendientes" ref="A1:R4" headerRowCount="1">
+  <autoFilter ref="A1:R4"/>
   <tableColumns count="18">
     <tableColumn id="1" name="archivo_pdf"/>
     <tableColumn id="2" name="ruta_pdf"/>
@@ -455,13 +455,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="82" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
@@ -573,12 +573,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>64-RD-0179-2026-11.pdf</t>
+          <t>64-RD-0185-2026-08.pdf</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0179-2026-11.pdf</t>
+          <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0185-2026-08.pdf</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -608,12 +608,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>0179-2026-ANA-AAA.MDD</t>
+          <t>0185-2026-ANA-AAA.MDD</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>179</t>
+          <t>185</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -623,7 +623,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>08/07/2026</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -633,27 +633,27 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>RD N° 0179-2026-ANA-AAA.MDD</t>
+          <t>RD N° 0185-2026-ANA-AAA.MDD</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>ARTÍCULO 1.- SANCIONAR al señor SANTIAGO JESUS MELENDEZ FLORES identificado con DNI N° 42708750, con una sanción administrativa de MULTA equivalente a diez coma cincuenta y nueve (10,59) UIT, por la infracción calificada como muy grave en materia de agua, por ocupar y desviar el cauce de la quebrada Virgen de la Candelaria producto del relleno con material de descarte producto de actividades de minería y/o lastre, sin autorización de la Autoridad Nacional del Agua.</t>
+          <t>ARTÍCULO 1.- ARCHIVAR el procedimiento administrativo sancionador iniciado contra la CORPORACIÓN INGENIEROS LAYAZU S.A.C., identificada con RUC N° 20600530951, por los fundamentos expresados en la parte considerativa de la presente resolución.</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>ARTÍCULO 1.- SANCIONAR al señor SANTIAGO JESUS MELENDEZ FLORES identificado con DNI N° 42708750, con una sanción administrativa de MULTA equivalente a diez coma cincuenta y nueve (10,59) UIT, por la infracción calificada como muy grave en materia de agua, por ocupar y desviar el cauce de la quebrada Virgen de la Candelaria producto del relleno con material de descarte producto de actividades de minería y/o lastre, sin autorización de la Autoridad Nacional del Agua.</t>
+          <t>ARTÍCULO 1.- ARCHIVAR el procedimiento administrativo sancionador iniciado contra la CORPORACIÓN INGENIEROS LAYAZU S.A.C., identificada con RUC N° 20600530951, por los fundamentos expresados en la parte considerativa de la presente resolución.</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>ARTÍCULO 2.- DISPONER que el depósito de la multa impuesta sea pagada mediante depósito en las agencias del Banco de la Nación en la Cuenta Corriente N° 0000-877174 de la Autoridad Nacional del Agua (concepto multas por infracción) en el plazo de quince (15) días hábiles de notificada la presente resolución, bajo apercibimiento de iniciarse la ejecución coactiva en caso de incumplimiento, debiendo alcanzar una copia del Boucher de depósito a la Administración Local de Agua Tambopata-Inambari dentro del tercer día de efectuado el mismo.</t>
+          <t>ARTÍCULO 2.- SANCIONAR a la MUNICIPALIDAD PROVINCIAL DE MANU, identificado con RUC N° 20162281845, con una MULTA equivalente a cero coma cinco (0,5) por la construcción de 02 estribos y aletones de concreto armado y la construcción de 02 pilas de concreto armado en los bienes naturales asociados al agua (ambas márgenes y cauce) de la quebrada Tazón, ubicado en el sector Machichi ubicado en el distrito de Huepetuhe, provincia de Manu, departamento de Madre de Dios.</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>ARTÍCULO 3.- DISPONER como Medida Complementaria, presente un plan de trabajo, a fin de restaurar a su estado natural el cauce de la quebrada Virgen de la Candelaria, en un plazo no mayor de sesenta (60) días calendarios, contados a partir del día siguiente de notificado con la presente resolución, conforme lo prevé el literal b, del artículo 25° de los Lineamientos para la tramitación del Procedimiento Administrativo Sancionador por transgresión a la Ley N° 29338, Ley de Recursos Hídricos y su Reglamento, aprobada mediante Resolución Jefatural N° 235- 2018-ANA, asumiendo el infractor los costos que demande su reposición.</t>
+          <t>ARTÍCULO 3.- DISPONER que el depósito de la multa impuesta sea pagada mediante depósito en las agencias del Banco de la Nación en la Cuenta Corriente N° 0000-877174 de la Autoridad Nacional del Agua (concepto multas por infracción) en el plazo de quince (15) días hábiles de notificado la presente resolución, bajo apercibimiento de iniciarse ejecución coactiva en caso de incumplimiento, debiendo alcanzar una copia del Boucher de depósito a la Administración Local de Agua Tambopata-Inambari dentro del tercer día de efectuado el mismo.</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -665,12 +665,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>64-RD-0180-2026-05.pdf</t>
+          <t>64-RD-0186-2026-05.pdf</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0180-2026-05.pdf</t>
+          <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0186-2026-05.pdf</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -700,12 +700,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>0180-2026-ANA-AAA.MDD</t>
+          <t>0186-2026-ANA-AAA.MDD</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>09/07/2026</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -725,30 +725,122 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>RD N° 0180-2026-ANA-AAA.MDD</t>
+          <t>RD N° 0186-2026-ANA-AAA.MDD</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>ARTICULO 1.- APROBAR los estudios de Huella Máxima que conforma el “Estudio de Delimitación de la Faja Marginal en un área de 10.23 ha de la Laguna Ananea, distrito de Quiaca, provincia de Sandia, departamento de Puno”, elaborado por la empresa CORI PUNO S.R.L. con RUC N° 20406339361, conforme a la metodología establecida en artículo 10 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales.</t>
+          <t>ARTÍCULO 1.- SANCIONAR al señor FRANKLIN ALFEREZ QUEA identificado con DNI N° 45513421, con una multa de cero coma noventa y uno (0,91) UIT, por la infracción calificada como leve en materia de agua, por utilizar el agua superficial de la quebrada Osjo Cachi con fines de uso minero, sin el correspondiente derecho de uso otorgado por la Autoridad Nacional del Agua, ubicada en el distrito de Ollachea, provincia de Carabaya, departamento de Puno.</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>ARTICULO 1.- APROBAR los estudios de Huella Máxima que conforma el “Estudio de Delimitación de la Faja Marginal en un área de 10.23 ha de la Laguna Ananea, distrito de Quiaca, provincia de Sandia, departamento de Puno”, elaborado por la empresa CORI PUNO S.R.L. con RUC N° 20406339361, conforme a la metodología establecida en artículo 10 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales.</t>
+          <t>ARTÍCULO 1.- SANCIONAR al señor FRANKLIN ALFEREZ QUEA identificado con DNI N° 45513421, con una multa de cero coma noventa y uno (0,91) UIT, por la infracción calificada como leve en materia de agua, por utilizar el agua superficial de la quebrada Osjo Cachi con fines de uso minero, sin el correspondiente derecho de uso otorgado por la Autoridad Nacional del Agua, ubicada en el distrito de Ollachea, provincia de Carabaya, departamento de Puno.</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>ARTÍCULO 2.- APROBAR a solicitud de parte, el ancho de la faja marginal de la Laguna Ananea con un ancho mínimo de 10.00 metros y un máximo de 35 metros, conforme a los alcances señalados en el artículo 4 y los criterios establecidos en el artículo 12 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales. La faja marginal está conformada por las áreas inmediatas superiores a la ribera de dichas fuentes de agua.</t>
+          <t>ARTÍCULO 2.- DISPONER que el depósito de la multa impuesta sea pagada mediante depósito en las agencias del Banco de la Nación en la Cuenta Corriente N° 0000-877174 de la Autoridad Nacional del Agua (concepto multas por infracción) en el plazo de quince (15) días hábiles de notificado la presente resolución, bajo apercibimiento de iniciarse ejecución coactiva en caso de incumplimiento, debiendo alcanzar una copia del Boucher de depósito a la Administración Local de Agua Tambopata-Inambari dentro del tercer día de efectuado el mismo.</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>ARTÍCULO 3.- APROBAR la delimitación de la faja marginal en la Laguna Ananea en un área de 10.23 ha, localizado en el sector de Untuca, distrito de Quiaca, provincia de Sandia, departamento de Puno, de conformidad a la metodología establecida en el artículo 6 y el procedimiento establecido en el artículo 18 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales, cuyo detalle se encuentra dispuesto en el anexo I y el plano que forman parte de la presente resolución.</t>
+          <t>ARTÍCULO 3.- DISPONER como Medida Complementaria el cese de la utilización ilegítima del recurso hídrico y otorgándole un plazo máximo de hasta tres (3) meses al señor Franklin Alferez Quea, computados a partir del día siguiente de la notificación de la presente resolución, para que regularice y obtenga el derecho de uso de agua correspondiente.</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>59-RD-0187-2026-05.pdf</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0187-2026-05.pdf</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>ALA Tahuamanu Madre de Dios</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>AAA Madre de Dios</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Resoluciones Emitidas por el ANA</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>De las Autoridades Administrativas del Agua</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>0187-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>09/07/2026</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00 am</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>RD N° 0187-2026-ANA-AAA.MDD</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- SANCIONAR a la señora PAULINA CRUZ MAMANI identificada con DNI N° 64035724, con una AMONESTACIÓN ESCRITA, por la infracción calificada como muy leve en materia de agua, por ocupar la ribera y faja marginal derecha del rio Madre de Dios sin la autorización correspondiente, ubicada en el sector Salvación, distrito y provincia de Manu, departamento de Madre de Dios.</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 1.- SANCIONAR a la señora PAULINA CRUZ MAMANI identificada con DNI N° 64035724, con una AMONESTACIÓN ESCRITA, por la infracción calificada como muy leve en materia de agua, por ocupar la ribera y faja marginal derecha del rio Madre de Dios sin la autorización correspondiente, ubicada en el sector Salvación, distrito y provincia de Manu, departamento de Madre de Dios.</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 2.- DISPONER como Medida Complementaria, que la imputada restaure la ribera y faja marginal derecha del río Madre de Dios al estado anterior a la infracción, debiendo de asumir los costos que demande su reposición y otorgarle a la imputada un plazo máximo de hasta tres (3) meses para que regularice y obtenga la autorización correspondiente, computados a partir del día siguiente de la notificación de la presente resolución.</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>ARTÍCULO 3.- DISPONER que la Administración Local de Agua Tahuamanu-Madre de Dios, verifique el cumplimiento de lo dispuesto en la Medida Complementaria.</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>

</xml_diff>

<commit_message>
chore: actualizar datos de carga - lote RDs 0209-0215 (7 publicadas)
Planilla regenerada con generar_planilla.py y preview de carga para el
lote 0213-0215 (3 RDs nuevas: 0213 obras minimas, 0214 sancion a Marcela
Ccama Lipa, 0215 sancion UPIS Isla de Brisas).
</commit_message>
<xml_diff>
--- a/data/resoluciones_pendientes.xlsx
+++ b/data/resoluciones_pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://autoridad-my.sharepoint.com/personal/ahuarancca_ana_gob_pe/Documents/MDD 2026/AAA/SubirPortal/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_81F32827CB731C30E6C839318AA1AB865CB189B5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3822144-49C2-4935-A447-0DA2D5D6829B}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_81F32827CB731C90E7350588270EC40657AB9987" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AB6C656-6A83-449F-8FBB-D57BE6DD1AC1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pendientes" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="55">
   <si>
     <t>archivo_pdf</t>
   </si>
@@ -81,10 +81,10 @@
     <t>articulo_elegido</t>
   </si>
   <si>
-    <t>64-RD-0200-2026-03.pdf</t>
-  </si>
-  <si>
-    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0200-2026-03.pdf</t>
+    <t>64-RD-0213-2026-04.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0213-2026-04.pdf</t>
   </si>
   <si>
     <t>64</t>
@@ -102,64 +102,67 @@
     <t>De las Autoridades Administrativas del Agua</t>
   </si>
   <si>
-    <t>0200-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>200</t>
+    <t>0213-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>213</t>
   </si>
   <si>
     <t>2026</t>
   </si>
   <si>
-    <t>22/07/2026</t>
+    <t>31/07/2026</t>
   </si>
   <si>
     <t>08:00:00 am</t>
   </si>
   <si>
-    <t>RD N° 0200-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 1° .- OTORGAR, licencia de uso de agua Superficial por un volumen hasta 4721.00 m³/año, para uso Poblacional, a favor de "JUNTA ADMINISTRADORA DE SERVICIO DE SANEAMIENTO (JASS) CHUMPIPAMPA", según el plano que forma parte de la presente resolución y.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 2.- INSCRIBIR la licencia otorgada mediante la presente resolución en el Registro Administrativo de Derechos de Uso de Agua.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 3.- REQUERIR a la JUNTA ADMINISTRADORA DE SERVICIO DE SANEAMIENTO (JASS) CHUMPIPAMPA, que presente la constancia de inscripción en el “Registro de Fuentes de Agua de Consumo Humano”, a cargo de la Autoridad de Salud competente, en un plazo máximo de treinta (30) días calendario, contados a partir del día siguiente de notificada la presente resolución.</t>
+    <t>RD N° 0213-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>PRIMERO. - AUTORIZAR al señor EMILIANO TAMAYO BERNALES, identificado con DNI N° 23961423, la ejecución de obras mínimas para trabajos de limpieza y descolmatación en el cauce de la quebrada Jayave, ubicado en la localidad de Virgen de la Candelaria, distrito de Inambari, provincia de Tambopata, región de Madre de Dios.</t>
+  </si>
+  <si>
+    <t>SEGUNDO.- PRECISAR que la ejecución de la obra mínima autorizada en el Artículo 1 de la presente resolución, tiene un plazo de treinta (30) días calendarios, computados a partir del día siguiente de notificada la presente resolución.</t>
+  </si>
+  <si>
+    <t>TERCERO.- DISPONER que la Administración Local de Agua Tambopata-Inambari realice una supervisión con la finalidad de corroborar el cumplimiento de la presente autorización.</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
-    <t>64-RD-0201-2026-03.pdf</t>
-  </si>
-  <si>
-    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0201-2026-03.pdf</t>
-  </si>
-  <si>
-    <t>0201-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>201</t>
-  </si>
-  <si>
-    <t>23/07/2026</t>
-  </si>
-  <si>
-    <t>RD N° 0201-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 1° .- OTORGAR, licencia de uso de agua Superficial por un volumen hasta 6445.00 m³/año, para uso Poblacional, a favor de "JUNTA ADMINISTRADORA DE SERVICIOS DE SANEAMIENTO (JASS) YANARCÓN-PHARA", según el plano que forma parte de la presente resolución y.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 3.- REQUERIR a la JUNTA ADMINISTRADORA DE SERVICIOS DE SANEAMIENTO (JASS) YANARCÓN-PHARA, que presente la constancia de inscripción en el “Registro de Fuentes de Agua de Consumo Humano”, a cargo de la Autoridad de Salud competente, en un plazo máximo de treinta (30) días calendario, contados a partir del día siguiente de notificada la presente resolución.</t>
-  </si>
-  <si>
-    <t>59-RD-0202-2026-03.pdf</t>
-  </si>
-  <si>
-    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0202-2026-03.pdf</t>
+    <t>64-RD-0214-2026-16.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0214-2026-16.pdf</t>
+  </si>
+  <si>
+    <t>0214-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>214</t>
+  </si>
+  <si>
+    <t>04/08/2026</t>
+  </si>
+  <si>
+    <t>RD N° 0214-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- DECLARAR FUNDADO EN PARTE el escrito de descargo interpuesto por la señora Marcela Ccama Lipa, conforme a los fundamentos expuestos en la parte considerativa de la presente resolución.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- SANCIONAR a la señora MARCELA CCAMA LIPA identificada con DNI N° 80588309 con una MULTA equivalente a doce coma cuarenta y seis (12,46) UIT, por la infracción calificada como muy grave en materia de agua, por efectuar vertimiento de aguas residuales en la quebrada Violeta, ubicada en el sector Violeta, distrito de Huepetuhe, provincia de Manu, departamento de Madre de Dios sin autorización de la Autoridad Nacional del Agua.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- DISPONER que el depósito de la multa impuesta sea pagada mediante depósito en las agencias del Banco de la Nación en la Cuenta Corriente N° 0000-877174 de la Autoridad Nacional del Agua (concepto multas por infracción) en el plazo de quince (15) días hábiles de notificado la presente resolución, bajo apercibimiento de iniciarse ejecución coactiva en caso de incumplimiento, debiendo alcanzar una copia del Boucher de depósito a la Administración Local de Agua Tambopata-Inambari dentro del tercer día de efectuado el mismo.</t>
+  </si>
+  <si>
+    <t>59-RD-0215-2026-12.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0215-2026-12.pdf</t>
   </si>
   <si>
     <t>59</t>
@@ -168,70 +171,22 @@
     <t>ALA Tahuamanu Madre de Dios</t>
   </si>
   <si>
-    <t>0202-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>202</t>
-  </si>
-  <si>
-    <t>24/07/2026</t>
-  </si>
-  <si>
-    <t>RD N° 0202-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 1.- DECLARAR la EXTINCIÓN de la licencia de uso de agua subterránea con fines productivos (otros usos), otorgada mediante la Resolución Directoral N° 0218- 2017-ANA/AAA-XIII MDD de fecha 17.08.2017, a favor de la empresa GRUPO AF S.A.C. con RUC N° 20601612209, por la causal prevista en el numeral 1 del artículo 70 de la Ley de Recursos Hídricos: Renuncia del titular.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 2.- REVERTIR al dominio del Estado, el volumen anual de 31 966,00 m 3, como consecuencia de la declaratoria de extinción de la licencia de uso de agua, proveniente de la fuente de agua subterránea.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 3.- INSCRIBIR el presente acto administrativo en el Registro Administrativo de Derechos de Uso de Agua (RADA).</t>
-  </si>
-  <si>
-    <t>64-RD-0203-2026-04.pdf</t>
-  </si>
-  <si>
-    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0203-2026-04.pdf</t>
-  </si>
-  <si>
-    <t>0203-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>203</t>
-  </si>
-  <si>
-    <t>RD N° 0203-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 1.- DECLARAR la EXTINCIÓN del Permiso de uso de agua atmosférico (lluvia), otorgado mediante Resolución Administrativa N° 0090-2019-ANA-AAA.MDD- ALA.TI de fecha 22.11.2019, a favor del Sr. Alipio Arnolio Poma Checalla, identificado con DNI N° 04811416, por la causal prevista en el numeral 1 del artículo 71 de la Ley de Recursos Hídricos: Muerte del titular del derecho.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 2.- REVERTIR al dominio del Estado, el volumen anual de 40,200.00 m³, como consecuencia de la declaratoria de extinción del permiso de uso de agua, proveniente de la fuente atmosférica (lluvia).</t>
-  </si>
-  <si>
-    <t>64-RD-0204-2026-03.pdf</t>
-  </si>
-  <si>
-    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0204-2026-03.pdf</t>
-  </si>
-  <si>
-    <t>0204-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>204</t>
-  </si>
-  <si>
-    <t>RD N° 0204-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 1°.- APROBAR la delimitación del Bloque “Comité de Usuarios de Agua Oqheyani Pampa”, según el plano que forma parte de la presente resolución, el cual tiene un área bajo riego de 2.50 hectáreas (ha.) y su centroide ubicado geográficamente en; 358588 metros(m)–Este(E) y 8 464 901 metros(m)–Norte(N), mediante el sistema de.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 2°.- OTORGAR, licencia de uso de agua Superficial por un volumen hasta 25021.00 m³/año, para uso Agrícola, a favor de "Comité de Usuarios de Agua Oqheyani Pampa".</t>
-  </si>
-  <si>
-    <t>ARTICULO 3º.- El titular de la licencia de uso de agua expedirá los Certificados Nominativos a sus asociados que acrediten la titularidad o posesión legítima del predio conformante del bloque; los que, a sola presentación a la Administración Local de Agua correspondiente, se inscriben en el Registro Administrativo de Derechos de Uso de Agua.</t>
+    <t>0215-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>215</t>
+  </si>
+  <si>
+    <t>RD N° 0215-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- SANCIONAR a la URBANIZACIÓN POPULAR DE INTERÉS SOCIAL (UPIS) ISLA DE BRISAS, con una MULTA equivalente a dos coma cero uno (2,01) UIT, por la infracción calificada como grave en materia de agua, por ocupar del humedal Campo Verde sin la autorización correspondiente, ubicada en el sector El Triunfo, distrito de Las Piedras, provincia de Tambopata, departamento de Madre de Dios.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- DISPONER que el depósito de la multa impuesta sea pagada mediante depósito en las agencias del Banco de la Nación en la Cuenta Corriente N° 0000-877174 de la Autoridad Nacional del Agua (concepto multas por infracción) en el plazo de quince (15) días hábiles de notificado la presente resolución, bajo apercibimiento de iniciarse ejecución coactiva en caso de incumplimiento, debiendo alcanzar una copia del Boucher de depósito a la Administración Local de Agua Tahuamanu-Madre de Dios dentro del tercer día de efectuado el mismo.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- DISPONER como Medida Complementaria que la UPIS Isla de Brisas, otorgándole un plazo máximo de hasta treinta (30) días calendarios, computados a partir del día siguiente de la notificación de la presente resolución, tome acciones orientadas a restaurar el cauce del humedal Campo Verde al estado anterior a la infracción, debiendo de asumir los costos que demande su reposición y se proceda con el retiro de las viviendas rusticas instaladas en el cauce del humedal Campo Verde que no hayan sido autorizadas por la Autoridad Nacional del Agua.</t>
   </si>
   <si>
     <t>2</t>
@@ -310,8 +265,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ResolucionesPendientes" displayName="ResolucionesPendientes" ref="A1:R6">
-  <autoFilter ref="A1:R6" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ResolucionesPendientes" displayName="ResolucionesPendientes" ref="A1:R4">
+  <autoFilter ref="A1:R4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="archivo_pdf"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ruta_pdf"/>
@@ -621,7 +576,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -696,7 +651,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
@@ -752,7 +707,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="105" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>35</v>
       </c>
@@ -799,27 +754,27 @@
         <v>41</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>34</v>
+        <v>43</v>
+      </c>
+      <c r="R3" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>22</v>
@@ -831,16 +786,16 @@
         <v>24</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>27</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>29</v>
@@ -862,118 +817,6 @@
       </c>
       <c r="R4" s="2" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="75" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="O5" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="P5" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q5" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="R5" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="O6" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="P6" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q6" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="R6" s="3" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: actualizar datos de carga - lote RDs 0216-0218 (3 publicadas)
</commit_message>
<xml_diff>
--- a/data/resoluciones_pendientes.xlsx
+++ b/data/resoluciones_pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://autoridad-my.sharepoint.com/personal/ahuarancca_ana_gob_pe/Documents/MDD 2026/AAA/SubirPortal/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_81F32827CB731C90E7350588270EC40657AB9987" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AB6C656-6A83-449F-8FBB-D57BE6DD1AC1}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_81F32827CB731C70E4679AFEF56FD40657AB9973" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41E25D40-1882-4DD8-B5F0-85EDE145C89A}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pendientes" sheetId="1" r:id="rId1"/>
@@ -81,10 +81,10 @@
     <t>articulo_elegido</t>
   </si>
   <si>
-    <t>64-RD-0213-2026-04.pdf</t>
-  </si>
-  <si>
-    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0213-2026-04.pdf</t>
+    <t>64-RD-0216-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0216-2026-03.pdf</t>
   </si>
   <si>
     <t>64</t>
@@ -102,67 +102,40 @@
     <t>De las Autoridades Administrativas del Agua</t>
   </si>
   <si>
-    <t>0213-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>213</t>
+    <t>0216-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>216</t>
   </si>
   <si>
     <t>2026</t>
   </si>
   <si>
-    <t>31/07/2026</t>
+    <t>05/08/2026</t>
   </si>
   <si>
     <t>08:00:00 am</t>
   </si>
   <si>
-    <t>RD N° 0213-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>PRIMERO. - AUTORIZAR al señor EMILIANO TAMAYO BERNALES, identificado con DNI N° 23961423, la ejecución de obras mínimas para trabajos de limpieza y descolmatación en el cauce de la quebrada Jayave, ubicado en la localidad de Virgen de la Candelaria, distrito de Inambari, provincia de Tambopata, región de Madre de Dios.</t>
-  </si>
-  <si>
-    <t>SEGUNDO.- PRECISAR que la ejecución de la obra mínima autorizada en el Artículo 1 de la presente resolución, tiene un plazo de treinta (30) días calendarios, computados a partir del día siguiente de notificada la presente resolución.</t>
-  </si>
-  <si>
-    <t>TERCERO.- DISPONER que la Administración Local de Agua Tambopata-Inambari realice una supervisión con la finalidad de corroborar el cumplimiento de la presente autorización.</t>
+    <t>RD N° 0216-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- APROBAR el.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- ACREDITAR la disponibilidad hídrica para el otorgamiento de derecho de uso de agua con fines de uso minero a favor de la ASOCIACIÓN DE MINEROS ARTESANALES ALTO MIRADOR con RUC N° 20542668394, para el proyecto denominado “Proyecto Minero Cumbre” ubicado en el sector Sisira, distrito de Alto Inambari, provincia de Sandia, departamento de Puno, cuya acreditación hídrica es de 10 805.00 m 3.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- PRECISAR que la presente acreditación de disponibilidad hídrica para el otorgamiento de derecho de uso de agua con fines de uso minero, tendrá un plazo máximo de vigencia de dos (2) años, la misma que se computará a partir del día siguiente de la notificación de la presente resolución.</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
-    <t>64-RD-0214-2026-16.pdf</t>
-  </si>
-  <si>
-    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0214-2026-16.pdf</t>
-  </si>
-  <si>
-    <t>0214-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>214</t>
-  </si>
-  <si>
-    <t>04/08/2026</t>
-  </si>
-  <si>
-    <t>RD N° 0214-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 1.- DECLARAR FUNDADO EN PARTE el escrito de descargo interpuesto por la señora Marcela Ccama Lipa, conforme a los fundamentos expuestos en la parte considerativa de la presente resolución.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 2.- SANCIONAR a la señora MARCELA CCAMA LIPA identificada con DNI N° 80588309 con una MULTA equivalente a doce coma cuarenta y seis (12,46) UIT, por la infracción calificada como muy grave en materia de agua, por efectuar vertimiento de aguas residuales en la quebrada Violeta, ubicada en el sector Violeta, distrito de Huepetuhe, provincia de Manu, departamento de Madre de Dios sin autorización de la Autoridad Nacional del Agua.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 3.- DISPONER que el depósito de la multa impuesta sea pagada mediante depósito en las agencias del Banco de la Nación en la Cuenta Corriente N° 0000-877174 de la Autoridad Nacional del Agua (concepto multas por infracción) en el plazo de quince (15) días hábiles de notificado la presente resolución, bajo apercibimiento de iniciarse ejecución coactiva en caso de incumplimiento, debiendo alcanzar una copia del Boucher de depósito a la Administración Local de Agua Tambopata-Inambari dentro del tercer día de efectuado el mismo.</t>
-  </si>
-  <si>
-    <t>59-RD-0215-2026-12.pdf</t>
-  </si>
-  <si>
-    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0215-2026-12.pdf</t>
+    <t>59-RD-0217-2026-12.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0217-2026-12.pdf</t>
   </si>
   <si>
     <t>59</t>
@@ -171,22 +144,49 @@
     <t>ALA Tahuamanu Madre de Dios</t>
   </si>
   <si>
-    <t>0215-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>215</t>
-  </si>
-  <si>
-    <t>RD N° 0215-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 1.- SANCIONAR a la URBANIZACIÓN POPULAR DE INTERÉS SOCIAL (UPIS) ISLA DE BRISAS, con una MULTA equivalente a dos coma cero uno (2,01) UIT, por la infracción calificada como grave en materia de agua, por ocupar del humedal Campo Verde sin la autorización correspondiente, ubicada en el sector El Triunfo, distrito de Las Piedras, provincia de Tambopata, departamento de Madre de Dios.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 2.- DISPONER que el depósito de la multa impuesta sea pagada mediante depósito en las agencias del Banco de la Nación en la Cuenta Corriente N° 0000-877174 de la Autoridad Nacional del Agua (concepto multas por infracción) en el plazo de quince (15) días hábiles de notificado la presente resolución, bajo apercibimiento de iniciarse ejecución coactiva en caso de incumplimiento, debiendo alcanzar una copia del Boucher de depósito a la Administración Local de Agua Tahuamanu-Madre de Dios dentro del tercer día de efectuado el mismo.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 3.- DISPONER como Medida Complementaria que la UPIS Isla de Brisas, otorgándole un plazo máximo de hasta treinta (30) días calendarios, computados a partir del día siguiente de la notificación de la presente resolución, tome acciones orientadas a restaurar el cauce del humedal Campo Verde al estado anterior a la infracción, debiendo de asumir los costos que demande su reposición y se proceda con el retiro de las viviendas rusticas instaladas en el cauce del humedal Campo Verde que no hayan sido autorizadas por la Autoridad Nacional del Agua.</t>
+    <t>0217-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>217</t>
+  </si>
+  <si>
+    <t>07/08/2026</t>
+  </si>
+  <si>
+    <t>RD N° 0217-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- SANCIONAR a la señora MONICA AROSQUIPA CALLAÑAUPA identificada con DNI N° 04817102, con una MULTA equivalente a cero coma cincuenta y cuatro (0,54) UIT, por la infracción calificada como grave en materia de agua, por ocupar la faja marginal derecha del rio Madre de Dios sin la autorización correspondiente, ubicada en el sector Puerto Rosario, distrito de y provincia de Tambopata, departamento de Madre de Dios.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- DISPONER que el depósito de la multa impuesta sea pagada mediante depósito en las agencias del Banco de la Nación en la Cuenta Corriente N° 0000-877174 de la Autoridad Nacional del Agua (concepto multas por infracción) en el plazo de quince (15) días hábiles de notificada la presente resolución, bajo apercibimiento de iniciarse la ejecución coactiva en caso de incumplimiento, debiendo alcanzar una copia del Boucher de depósito a la Administración Local de Agua Tahuamanu-Madre de Dios dentro del tercer día de efectuado el mismo.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- DISPONER como Medida Complementaria que la señora Mónica Arosquipa Callañaupa, otorgándole un plazo máximo de hasta treinta (30) días calendarios, computados a partir del día siguiente de la notificación de la presente resolución, tome acciones orientadas a el retiro de las obras ejecutadas (vivienda) del bien asociado ubicado en la margen derecha del rio Madre de Dios, por no contar con la autorización correspondiente, la Autoridad Nacional del Agua en coordinación con los Gobiernos Locales y Defensa Civil promoverán mecanismos de reubicación de poblaciones asentadas.</t>
+  </si>
+  <si>
+    <t>64-RD-0218-2026-04.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0218-2026-04.pdf</t>
+  </si>
+  <si>
+    <t>0218-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>218</t>
+  </si>
+  <si>
+    <t>RD N° 0218-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- AUTORIZAR la ocupación futura de la faja marginal en la margen izquierda del río Malinowsky, destinadas a la implementación temporal de la Base Militar Fátima y un helipuerto, a favor de la 2DA BRIGADA DE PROTECCION DE LA AMAZONIA DEL EJERCITO DEL PERU con RUC N° 20131369124; dicha área se ubica en el sector Malinowski, distrito de Inambari, provincia de Tambopata y departamento de Madre de Dios; por un plazo máximo de dos (2) años, computado a partir del día siguiente de la notificación de la presente resolución.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- REGISTRAR la presente autorización en el inventario de áreas ocupadas de las fajas marginales de fuentes naturales de agua, en cumplimiento de lo establecido en el artículo 5 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- PRECISAR que la presente resolución no autoriza la tala de recursos forestales ni la quema de bosques, actividades que están reguladas en la Ley N° 29763, Ley Forestal y de Fauna Silvestre, y sus Reglamentos.</t>
   </si>
   <si>
     <t>2</t>
@@ -651,7 +651,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
@@ -703,11 +703,11 @@
       <c r="Q2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="R2" s="2" t="s">
-        <v>34</v>
+      <c r="R2" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="105" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="120" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>35</v>
       </c>
@@ -715,10 +715,10 @@
         <v>36</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>22</v>
@@ -730,51 +730,51 @@
         <v>24</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>27</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>29</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="R3" s="3" t="s">
-        <v>54</v>
+        <v>45</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:18" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>22</v>
@@ -795,7 +795,7 @@
         <v>27</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
chore: actualizar datos de carga - lote RDs 0219-0236 (18 publicadas)
</commit_message>
<xml_diff>
--- a/data/resoluciones_pendientes.xlsx
+++ b/data/resoluciones_pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://autoridad-my.sharepoint.com/personal/ahuarancca_ana_gob_pe/Documents/MDD 2026/AAA/SubirPortal/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_81F32827CB731C70E4679AFEF56FD40657AB9973" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41E25D40-1882-4DD8-B5F0-85EDE145C89A}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_81F32827CB731C10EE126DAD7C67B3067ABAE02C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE376E2B-9D47-455A-86E8-6A7CE812188D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="5550" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pendientes" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="173">
   <si>
     <t>archivo_pdf</t>
   </si>
@@ -81,10 +81,10 @@
     <t>articulo_elegido</t>
   </si>
   <si>
-    <t>64-RD-0216-2026-03.pdf</t>
-  </si>
-  <si>
-    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0216-2026-03.pdf</t>
+    <t>64-RD-0219-2026-05.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0219-2026-05.pdf</t>
   </si>
   <si>
     <t>64</t>
@@ -102,40 +102,67 @@
     <t>De las Autoridades Administrativas del Agua</t>
   </si>
   <si>
-    <t>0216-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>216</t>
+    <t>0219-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>219</t>
   </si>
   <si>
     <t>2026</t>
   </si>
   <si>
-    <t>05/08/2026</t>
+    <t>10/08/2026</t>
   </si>
   <si>
     <t>08:00:00 am</t>
   </si>
   <si>
-    <t>RD N° 0216-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 1.- APROBAR el.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 2.- ACREDITAR la disponibilidad hídrica para el otorgamiento de derecho de uso de agua con fines de uso minero a favor de la ASOCIACIÓN DE MINEROS ARTESANALES ALTO MIRADOR con RUC N° 20542668394, para el proyecto denominado “Proyecto Minero Cumbre” ubicado en el sector Sisira, distrito de Alto Inambari, provincia de Sandia, departamento de Puno, cuya acreditación hídrica es de 10 805.00 m 3.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 3.- PRECISAR que la presente acreditación de disponibilidad hídrica para el otorgamiento de derecho de uso de agua con fines de uso minero, tendrá un plazo máximo de vigencia de dos (2) años, la misma que se computará a partir del día siguiente de la notificación de la presente resolución.</t>
+    <t>RD N° 0219-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- APROBAR el caudal ecológico del rio Araza equivalente a un volumen anual de hasta 28 089 245 m3, siendo el volumen de agua que debe mantenerse para la protección y conservación de la fuente natural y los ecosistemas involucrados.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- ACREDITAR la disponibilidad hídrica para el otorgamiento de derecho de uso de agua superficial con fines de uso energético a favor la MUNICIPALIDAD DISTRITAL DE MARCAPATA con RUC N° 20214061474 para el proyecto denominado “Ampliación del Servicio de Energía Eléctrica Mediante Minicentral Hidroeléctrica de 1 MW, en el C.P. de Amacho, distrito de Marcapata, provincia de Quispicanchi, región Cusco”, ubicado en el centro poblado de Amacho, distrito de Marcapata, provincia de Quispicanchi, departamento de Cusco, cuya acreditación hídrica anual es hasta 39 420 000 m3.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- PRECISAR que la presente acreditación de disponibilidad hídrica para el otorgamiento de derecho de uso de agua superficial con fines de uso energético, tendrá un plazo máximo de vigencia de dos (2) años, la misma que se computará a partir del día siguiente de la notificación de la presente resolución.</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
-    <t>59-RD-0217-2026-12.pdf</t>
-  </si>
-  <si>
-    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0217-2026-12.pdf</t>
+    <t>64-RD-0220-2026-14.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0220-2026-14.pdf</t>
+  </si>
+  <si>
+    <t>0220-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>220</t>
+  </si>
+  <si>
+    <t>11/08/2026</t>
+  </si>
+  <si>
+    <t>RD N° 0220-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- SANCIONAR a la empresa MINERA SECA AGUAJAL S.A., identificada con RUC N° 20528082786 con una MULTA equivalente a veinte coma cuarenta y ocho (20,48) UIT, por la infracción calificada como muy grave en materia de agua, por efectuar vertimiento de aguas residuales de tipo minero en la quebrada Sin Nombre sin autorización de la Autoridad Nacional del Agua.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- DISPONER que el depósito de la multa impuesta sea pagada mediante depósito en las agencias del Banco de la Nación en la Cuenta Corriente N° 0000-877174 de la Autoridad Nacional del Agua (concepto multas por infracción) en el plazo de quince (15) días hábiles de notificado la presente resolución, bajo apercibimiento de iniciarse ejecución coactiva en caso de incumplimiento, debiendo alcanzar una copia del Boucher de depósito a la Administración Local de Agua Tambopata-Inambari dentro del tercer día de efectuado el mismo.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- DISPONER como Medida Complementaria, el cese inmediato del vertimiento de aguas residuales de tipo minero en la quebrada Sin Nombre y realice los trámites necesarios para obtener la autorización de vertimiento de aguas residuales industriales tratadas como medida complementaria, otorgándole a la empresa sancionada un plazo máximo de hasta treinta (30) días calendarios, computados a partir de la notificación con la presente resolución.</t>
+  </si>
+  <si>
+    <t>59-RD-0221-2026-07.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0221-2026-07.pdf</t>
   </si>
   <si>
     <t>59</t>
@@ -144,49 +171,376 @@
     <t>ALA Tahuamanu Madre de Dios</t>
   </si>
   <si>
-    <t>0217-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>217</t>
-  </si>
-  <si>
-    <t>07/08/2026</t>
-  </si>
-  <si>
-    <t>RD N° 0217-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 1.- SANCIONAR a la señora MONICA AROSQUIPA CALLAÑAUPA identificada con DNI N° 04817102, con una MULTA equivalente a cero coma cincuenta y cuatro (0,54) UIT, por la infracción calificada como grave en materia de agua, por ocupar la faja marginal derecha del rio Madre de Dios sin la autorización correspondiente, ubicada en el sector Puerto Rosario, distrito de y provincia de Tambopata, departamento de Madre de Dios.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 2.- DISPONER que el depósito de la multa impuesta sea pagada mediante depósito en las agencias del Banco de la Nación en la Cuenta Corriente N° 0000-877174 de la Autoridad Nacional del Agua (concepto multas por infracción) en el plazo de quince (15) días hábiles de notificada la presente resolución, bajo apercibimiento de iniciarse la ejecución coactiva en caso de incumplimiento, debiendo alcanzar una copia del Boucher de depósito a la Administración Local de Agua Tahuamanu-Madre de Dios dentro del tercer día de efectuado el mismo.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 3.- DISPONER como Medida Complementaria que la señora Mónica Arosquipa Callañaupa, otorgándole un plazo máximo de hasta treinta (30) días calendarios, computados a partir del día siguiente de la notificación de la presente resolución, tome acciones orientadas a el retiro de las obras ejecutadas (vivienda) del bien asociado ubicado en la margen derecha del rio Madre de Dios, por no contar con la autorización correspondiente, la Autoridad Nacional del Agua en coordinación con los Gobiernos Locales y Defensa Civil promoverán mecanismos de reubicación de poblaciones asentadas.</t>
-  </si>
-  <si>
-    <t>64-RD-0218-2026-04.pdf</t>
-  </si>
-  <si>
-    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0218-2026-04.pdf</t>
-  </si>
-  <si>
-    <t>0218-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>218</t>
-  </si>
-  <si>
-    <t>RD N° 0218-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 1.- AUTORIZAR la ocupación futura de la faja marginal en la margen izquierda del río Malinowsky, destinadas a la implementación temporal de la Base Militar Fátima y un helipuerto, a favor de la 2DA BRIGADA DE PROTECCION DE LA AMAZONIA DEL EJERCITO DEL PERU con RUC N° 20131369124; dicha área se ubica en el sector Malinowski, distrito de Inambari, provincia de Tambopata y departamento de Madre de Dios; por un plazo máximo de dos (2) años, computado a partir del día siguiente de la notificación de la presente resolución.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 2.- REGISTRAR la presente autorización en el inventario de áreas ocupadas de las fajas marginales de fuentes naturales de agua, en cumplimiento de lo establecido en el artículo 5 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 3.- PRECISAR que la presente resolución no autoriza la tala de recursos forestales ni la quema de bosques, actividades que están reguladas en la Ley N° 29763, Ley Forestal y de Fauna Silvestre, y sus Reglamentos.</t>
+    <t>0221-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>221</t>
+  </si>
+  <si>
+    <t>RD N° 0221-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- SANCIONAR a la UNIDAD EJECUTORA 1392 – SUB REGIÓN MANU identificada con RUC N° 20490448951, con una MULTA equivalente a dos coma cero uno (2,01) UIT, por ejecutar obras del proyecto denominado “Mejoramiento y Ampliación del Sistema de Agua Potable y Saneamiento Básico en los Centros Poblados de Puerto Azul e Isla de los Valles, Distrito de Fitzcarrald - Manu - Madre de Dios”, que consiste en una infraestructura de aprovechamiento de captación de agua de una fuente subterránea (pozo mixto), una caseta de control y un reservorio elevado de almacenamiento de agua, ubicadas en la comunidad nativa Puerto Azul, distrito de Fitzcarrald, provincia de Manu, departamento Madre de Dios.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- DISPONER que el depósito de la multa impuesta sea pagada mediante depósito en las agencias del Banco de la Nación en la Cuenta Corriente N° 0000-877174 de la Autoridad Nacional del Agua (concepto multas por infracción) en el plazo de quince (15) días hábiles de notificado la presente resolución, bajo apercibimiento de iniciarse ejecución coactiva en caso de incumplimiento, debiendo alcanzar una copia del Boucher de depósito a la Administración Local de Agua Tahuamanu-Madre de Dios dentro del tercer día de efectuado el mismo.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- DISPONER como Medida Complementaria, otorgarle a la imputada un plazo máximo de hasta treinta (30) días calendarios, computados a partir del día siguiente de la notificación de la presente resolución, para que regularice y obtenga la autorización correspondiente.</t>
+  </si>
+  <si>
+    <t>64-RD-0222-2026-12.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0222-2026-12.pdf</t>
+  </si>
+  <si>
+    <t>0222-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>222</t>
+  </si>
+  <si>
+    <t>RD N° 0222-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- SANCIONAR a la empresa JUANITA DOS MIL S.R.L. identificada con RUC N° 20490561251, con una MULTA equivalente a doce coma catorce (12,14) UIT, por la infracción calificada como muy grave en materia de agua, por efectuar vertimiento de aguas residuales de tipo minero en la margen izquierda de la quebrada Aguajal sin autorización de la Autoridad Nacional del Agua.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- DISPONER como Medida Complementaria, el cese inmediato del vertimiento de aguas residuales de tipo minero en la margen izquierda de la quebrada Aguajal y realice los trámites necesarios para obtener la autorización de vertimiento de aguas residuales industriales tratadas como medida complementaria, otorgándole a la empresa sancionada un plazo máximo de seis (6) meses, para obtener dicha autorización, computados a partir de la notificación con la presente resolución.</t>
+  </si>
+  <si>
+    <t>64-RD-0223-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0223-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>0223-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>223</t>
+  </si>
+  <si>
+    <t>13/08/2026</t>
+  </si>
+  <si>
+    <t>RD N° 0223-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1°.- APROBAR la delimitación del Bloque COMITÉ DE USUARIOS CANAL DE RIEGO ICHANI, según el plano que forma parte de la presente resolución, el cual tiene un área bajo riego de 20.00 hectáreas (ha) y su centroide ubicado geográficamente en 447 553 metros (m)-Este (E) y 8409854 metros (m)-Norte (N) mediante el sistema de.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2°.- OTORGAR, licencia de uso de agua Superficial por un volumen hasta 61494.00 m³/año, para uso Agrícola, a favor de " COMITÉ DE USUARIOS CANAL DE RIEGO ICHANI ".</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3°.- El titular de la licencia de uso de agua expedirá los Certificados Nominativos a sus asociados que acrediten la titularidad o posesión legítima del predio conformante del bloque; los que a sola presentación a la Administración Local de Agua Tambopata-Inambari, se inscriben en el Registro Administrativo de Derechos de Uso de Agua.</t>
+  </si>
+  <si>
+    <t>59-RD-0224-2026-05.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0224-2026-05.pdf</t>
+  </si>
+  <si>
+    <t>0224-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>224</t>
+  </si>
+  <si>
+    <t>14/08/2026</t>
+  </si>
+  <si>
+    <t>RD N° 0224-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- SANCIONAR al señor CECILIO FERNANDEZ ORTIZ identificado con DNI N° 05061388, con una AMONESTACIÓN ESCRITA, por la infracción calificada como leve en materia de agua, por utilizar el agua subterránea con fines de uso doméstico-poblacional, sin el correspondiente derecho de uso otorgado por la Autoridad Nacional del Agua en la unidad operativa vivienda ubicado en la localidad de Iberia, distrito de Iberia, provincia de Tahuamanu, departamento de Madre de Dios.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- INSCRIBIR en el Registro de Sanciones, la sanción impuesta en el artículo 1, una vez que quede consentida o agote la vía administrativa.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- NOTIFICAR la presente resolución al señor Cecilio Fernández Ortiz en su domicilio; poner de conocimiento a la Administración Local de Agua Tahuamanu-Madre de Dios; y disponer su publicación en el portal web institucional de la Autoridad Nacional del Agua: www.ana.gob.pe.</t>
+  </si>
+  <si>
+    <t>59-RD-0225-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0225-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>0225-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>225</t>
+  </si>
+  <si>
+    <t>RD N° 0225-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- DECLARAR IMPROCEDENTE la solicitud presentada por el señor MARIO RAMOS SALAS identificado con DNI N° 25317903, sobre la autorización de ejecución de obras de servicios públicos (servicios higiénicos o baños públicos) en la faja marginal ubicada en el distrito de Laberinto, provincia de Tambopata, departamento de Madre de Dios, por los fundamentos expuestos en la parte considerativa de la presente resolución.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- DISPONER el ARCHIVAMIENTO DEFINITIVO del expediente administrativo una vez vencido los plazos recursivos.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- NOTIFICAR la presente resolución al señor Mario Ramos Salas en su domicilio; poner de conocimiento a la Administración Local de Agua Tahuamanu-Madre de Dios; y disponer su publicación en el portal web institucional de la Autoridad Nacional del Agua: www.ana.gob.pe.</t>
+  </si>
+  <si>
+    <t>59-RD-0226-2026-04.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0226-2026-04.pdf</t>
+  </si>
+  <si>
+    <t>0226-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>226</t>
+  </si>
+  <si>
+    <t>RD N° 0226-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- DECLARAR IMPROCEDENTE la solicitud presentada por la ASOCIACIÓN DE PESCADORES ARTESANALES DE PUERTO MALDONADO con RUC N° 20527604291, sobre la autorización de ocupación y ejecución de obras de servicios públicos (embarcadero fluvial) en la faja marginal, ubicada en el distrito de Tambopata, provincia de Tambopata, departamento de Madre de Dios, por los fundamentos expuestos en la parte considerativa de la presente resolución.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- NOTIFICAR la presente resolución a la Asociación de Pescadores Artesanales de Puerto Maldonado en su domicilio; poner de conocimiento a la Administración Local de Agua Tahuamanu-Madre de Dios; y disponer su publicación en el portal web institucional de la Autoridad Nacional del Agua: www.ana.gob.pe.</t>
+  </si>
+  <si>
+    <t>59-RD-0227-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0227-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>0227-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>227</t>
+  </si>
+  <si>
+    <t>RD N° 0227-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- ACREDITAR la disponibilidad hídrica para el otorgamiento de derecho de uso de agua con fines de uso poblacional a favor la empresa CONSTRUCTORA E INVERSIONES BRAGANZA S.A.C. con RUC N° 20609090431, para el desarrollo del proyecto denominado “Mi vivienda techo propio, fondo que impulsa el estado peruano, a través del Ministerio de Vivienda y Construcción, ubicado en el sector de Bello Horizonte, distrito de Las Piedras, provincia de Tambopata, departamento de Madre de Dios”, cuya acreditación hídrica es de 61495.00 m3.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- PRECISAR que la presente acreditación de disponibilidad hídrica para el otorgamiento de derecho de uso de agua con fines de uso poblacional, tendrá un plazo máximo de vigencia de dos (2) años, la misma que se computará a partir del día siguiente de la notificación de la presente resolución.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- PRECISAR que la presente acreditación de disponibilidad hídrica para el otorgamiento de derecho de uso de agua con fines de uso poblacional, no autoriza la ejecución de obras ni la utilización del recurso hídrico.</t>
+  </si>
+  <si>
+    <t>59-RD-0228-2026-04.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0228-2026-04.pdf</t>
+  </si>
+  <si>
+    <t>0228-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>228</t>
+  </si>
+  <si>
+    <t>17/08/2026</t>
+  </si>
+  <si>
+    <t>RD N° 0228-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- ACREDITAR la disponibilidad hídrica para el otorgamiento de derecho de uso de agua con fines de uso industrial a favor de la COMUNIDAD NATIVA LA VICTORIA con RUC Nº 20613162934, para el desarrollo del proyecto denominado “Optimización de los procesos de recolección y transformación primaria de la Almendra de Huicungo, asegurando el uso sostenible del bosque bajo la activa participación de las mujeres de la Comunidad Nativa La Victoria, Tambopata, Madre de Dios”, cuya acreditación hídrica es de 270 m 3/año.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- PRECISAR que la presente acreditación de disponibilidad hídrica para el otorgamiento de derecho de uso de agua con fines de uso industrial, tendrá un plazo máximo de vigencia de dos (2) años, la misma que se computará a partir del día siguiente de la notificación de la presente resolución.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- PRECISAR que la presente acreditación de disponibilidad hídrica para el otorgamiento de derecho de uso de agua con fines de uso industrial, no autoriza la ejecución de obras ni la utilización del recurso hídrico.</t>
+  </si>
+  <si>
+    <t>59-RD-0229-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0229-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>0229-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>229</t>
+  </si>
+  <si>
+    <t>RD N° 0229-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- OTORGAR autorización de uso temporal de un área de la faja marginal izquierda del rio Tambopata para siembra de cultivos de 0.80 hectáreas (ha), a favor de la señora VALENZUELA SALAZAR, HEYDY DAMARIS identificada con DNI N° 43549278; dicha área se ubica en el sector Chonta, distrito y provincia de Tambopata, departamento de Madre de Dios.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- PRECISAR que la presente autorización tiene un plazo de vigencia de tres (3) años, la misma que se computará a partir de la fecha de emisión de la presente resolución.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- REGISTRAR la presente autorización en el inventario de áreas ocupadas de las fajas marginales de fuentes naturales de agua, en cumplimiento de lo establecido en el artículo 5 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales.</t>
+  </si>
+  <si>
+    <t>59-RD-0230-2026-08.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0230-2026-08.pdf</t>
+  </si>
+  <si>
+    <t>0230-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>230</t>
+  </si>
+  <si>
+    <t>21/08/2026</t>
+  </si>
+  <si>
+    <t>RD N° 0230-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- SANCIONAR a la señora CONSTANTINA CARITA LÓPEZ identificada con DNI N° 04808544, con una MULTA equivalente a cero coma sesenta y uno (0,61) UIT, por la infracción calificada como leve en materia de agua, por desviar el cauce de la quebrada Huayrurochayoc sin la autorización correspondiente, ubicado en el distrito Huepetuhe, provincia de Manu, departamento de Madre de Dios.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- DISPONER como Medida Complementaria, que la imputada restaure el cauce de la quebrada Huayrurochayoc al estado anterior a la infracción, debiendo de asumir los costos que demande su reposición en un plazo de treinta (30) días hábiles, computados a partir del día siguiente de la notificación de la presente resolución.</t>
+  </si>
+  <si>
+    <t>59-RD-0231-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0231-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>0231-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>231</t>
+  </si>
+  <si>
+    <t>24/08/2026</t>
+  </si>
+  <si>
+    <t>RD N° 0231-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- OTORGAR autorización de uso temporal de un área de la bifurcación derecha del rio Madre de Dios para siembra de cultivos, en un área de 2.55 hectáreas (ha), a favor del señor MERCADO CHALLCO, ELIAS ANGEL identificado con DNI N° 42111809; dicha área se ubica en el sector Adán Rayo, distrito y provincia de Manu, departamento de Madre de Dios.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- PRECISAR que la presente autorización tiene un plazo de vigencia de cuatro (4) años, la misma que se computará a partir de la fecha de emisión de la presente resolución.</t>
+  </si>
+  <si>
+    <t>64-RD-0232-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0232-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>0232-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>232</t>
+  </si>
+  <si>
+    <t>RD N° 0232-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- OTORGAR autorización de uso temporal de un área de la bifurcación izquierda del rio Inambari para siembra de cultivos, en un área de 5.00 hectáreas (ha), a favor del señor CONDORI CHAVEZ, LUCIANO identificado con DNI N° 42874557; dicha área se ubica en el sector Ponal, distrito de Inambari, provincia de Tambopata, departamento de Madre de Dios.</t>
+  </si>
+  <si>
+    <t>64-RD-0233-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0233-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>0233-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>233</t>
+  </si>
+  <si>
+    <t>RD N° 0233-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- OTORGAR autorización de uso temporal de un área de la bifurcación izquierda del rio Inambari para siembra de cultivos, en un área de 4.70 hectáreas (ha), a favor de la señora HUAMAN CHAVEZ, ALEJA identificada con DNI N° 24488309; dicha área se ubica en el sector Ponal, distrito de Inambari, provincia de Tambopata, departamento de Madre de Dios.</t>
+  </si>
+  <si>
+    <t>59-RD-0234-2026-05.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0234-2026-05.pdf</t>
+  </si>
+  <si>
+    <t>0234-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>234</t>
+  </si>
+  <si>
+    <t>25/08/2026</t>
+  </si>
+  <si>
+    <t>RD N° 0234-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- ACREDITAR la disponibilidad hídrica superficial en vía de regularización con fines de uso acuícola, a favor del del “Instituto de Investigaciones de la Amazonia Esta es una copia auténtica imprimible de un documento electrónico archivado de ANA, aplicando lo dispuesto por el Art. 25 de D.S 070-2013-PCM y la Tercera Disposición Complementaria Final del D.S 026-2016-PCM. Su autenticidad e integridad pueden ser contrastadas a través de: https://sisged.ana.gob.pe/consultas e ingresando la siguiente clave : 3C21A2FD Peruana-IIAP”, identificado con RUC N° 20171781648, cuya acreditación hídrica es de 103 740.00 m3/año.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- APROBAR el caudal ecológico en vía de regularización de la Quebrada El Castañal, estableciendo un volumen anual de 122,101.16 m 3 /año.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- APROBAR el plan de aprovechamiento hídrico, así como el sistema hidráulico y AUTORIZAR la ejecución de obras de aprovechamiento hídrico superficial en vía de regularización conforme a las características señaladas en la Formato N° 03, planos adjuntos y verificación técnica de campo a favor del administrado.</t>
+  </si>
+  <si>
+    <t>64-RD-0235-2026-04.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0235-2026-04.pdf</t>
+  </si>
+  <si>
+    <t>0235-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>235</t>
+  </si>
+  <si>
+    <t>26/08/2026</t>
+  </si>
+  <si>
+    <t>RD N° 0235-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- OTORGAR, Autorización de Uso de Agua superficial para la ejecución de obras para el proyecto denominado "Mejoramiento del camino vecinal Aymaña-Pallca, pampa- Lacaya-Puna, Apacheta-Quichu en los distritos de Ollachea y Corani de la provincia Carabaya- departamento de Puno”, a favor de la empresa GRUPO FER CONS S.A.C. identificado con RUC N° 20447689503, cuyo aprovechamiento de agua será por un volumen de hasta 43 519.68 m3.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- PRECISAR que la presente resolución tendrá un plazo de vigencia de doce (12) meses que se computará a partir del día siguiente de la notificación de la presente resolución.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- INSCRIBIR el presente acto administrativo en el Registro Administrativo de Derechos de Uso de Agua (RADA).</t>
+  </si>
+  <si>
+    <t>64-RD-0236-2026-04.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0236-2026-04.pdf</t>
+  </si>
+  <si>
+    <t>0236-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>236</t>
+  </si>
+  <si>
+    <t>RD N° 0236-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- OTORGAR, Autorización de Uso de Agua superficial para la ejecución de obras para el proyecto denominado “Mejoramiento del camino Departamental MD-101 tramo: EMP. PE-30C (Santa Rosa) - Puerto Carlos, Distrito de Inambari - Provincia de Tambopata - Departamento de Madre de Dios”, a favor de la Dirección Regional de Transportes y Comunicaciones del Gobierno Regional Madre de Dios con RUC N° 20527143200, cuyo aprovechamiento de agua será por un volumen de hasta 5 346.48 m 3.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- PRECISAR que la presente resolución tendrá un plazo de vigencia de dos (2) meses que se computará a partir del día siguiente de la notificación de la presente resolución.</t>
   </si>
   <si>
     <t>2</t>
@@ -265,8 +619,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ResolucionesPendientes" displayName="ResolucionesPendientes" ref="A1:R4">
-  <autoFilter ref="A1:R4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ResolucionesPendientes" displayName="ResolucionesPendientes" ref="A1:R19">
+  <autoFilter ref="A1:R19" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="archivo_pdf"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ruta_pdf"/>
@@ -576,8 +930,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:R19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="82" customWidth="1"/>
@@ -595,7 +949,7 @@
     <col min="18" max="18" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -651,7 +1005,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
@@ -704,10 +1058,10 @@
         <v>33</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>54</v>
+        <v>172</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="120" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="87" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>35</v>
       </c>
@@ -715,10 +1069,10 @@
         <v>36</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>22</v>
@@ -730,51 +1084,51 @@
         <v>24</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>27</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>29</v>
       </c>
       <c r="M3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="P3" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="P3" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>45</v>
       </c>
       <c r="R3" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="105" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="116" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>22</v>
@@ -795,7 +1149,7 @@
         <v>27</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>29</v>
@@ -816,6 +1170,846 @@
         <v>53</v>
       </c>
       <c r="R4" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="87" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q5" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="58" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q6" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="R6" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="87" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q7" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="R7" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="R8" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="87" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="O9" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="R9" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="87" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q10" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="R10" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="87" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="O11" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="Q11" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="R11" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="58" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="O12" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="P12" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="Q12" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="R12" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="87" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="O13" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="P13" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q13" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="R13" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="58" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="O14" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q14" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="R14" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="58" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="O15" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="Q15" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="R15" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="58" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="Q16" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="R16" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="P17" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q17" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="R17" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="O18" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="P18" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q18" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="R18" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="87" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="N19" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="O19" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="P19" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="Q19" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="R19" s="2" t="s">
         <v>34</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar datos de carga - lote RDs 0249-0253 (5 publicadas)
</commit_message>
<xml_diff>
--- a/data/resoluciones_pendientes.xlsx
+++ b/data/resoluciones_pendientes.xlsx
@@ -1,26 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://autoridad-my.sharepoint.com/personal/ahuarancca_ana_gob_pe/Documents/MDD 2026/AAA/SubirPortal/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_81F3282764239F759965B268853852C65733ADEB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E45D5446-8329-4A8F-9370-E7DA5ED121E5}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_81F32827CB731C30E981E03EE380B3865CB177D2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65FF975F-7FFC-4CC9-845E-FC2ED28244B5}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="5550" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pendientes" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="69">
   <si>
     <t>archivo_pdf</t>
   </si>
@@ -76,10 +81,10 @@
     <t>articulo_elegido</t>
   </si>
   <si>
-    <t>59-RD-0248-2026-04.pdf</t>
-  </si>
-  <si>
-    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0248-2026-04.pdf</t>
+    <t>59-RD-0249-2026-07.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0249-2026-07.pdf</t>
   </si>
   <si>
     <t>59</t>
@@ -97,10 +102,13 @@
     <t>De las Autoridades Administrativas del Agua</t>
   </si>
   <si>
-    <t>0248-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>248</t>
+    <t>0249-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>249</t>
+  </si>
+  <si>
+    <t>2026</t>
   </si>
   <si>
     <t>02/09/2026</t>
@@ -109,19 +117,121 @@
     <t>08:00:00 am</t>
   </si>
   <si>
-    <t>RD N° 0248-2026-ANA-AAA.MDD</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 1.- APROBAR los estudios de huella máxima que conforma el estudio técnico denominado “Delimitación de la Faja Marginal de la Quebrada 28 de Julio, en el Sector Nuevo San Martin, ubicado en el distrito y provincia de Tahuamanu, departamento Madre de Dios”, presentada a solicitud de parte, conforme a la metodología establecida en artículo 10 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 2.- APROBAR a solicitud de parte, el ancho de la faja marginal de la quebrada 28 de Julio en un tramo de 263 metros (m), un ancho mínimo de 6.00 m y un máximo de 9.00 m en la margen derecha y un ancho mínimo de 5.00 m y un máximo de 7.00 m en la margen izquierda, conforme a los alcances señalados en el artículo 4 y los criterios establecidos en el artículo 12 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales.</t>
-  </si>
-  <si>
-    <t>ARTÍCULO 3.- APROBAR la delimitación de la faja marginal en el tramo materia de estudio de la quebrada 28 de Julio, ubicada en el sector Nuevo San Martín, distrito y provincia de Tahuamanu, departamento de Madre de Dios, de conformidad a la metodología establecida en el artículo 6 y el procedimiento establecido en el artículo 18 del Reglamento para la Delimitación y Mantenimiento de Fajas Marginales, cuyo detalle se encuentra dispuesto en el plano que forman parte de la presente resolución.</t>
+    <t>RD N° 0249-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- SANCIONAR a la empresa NICONSTA COMPAÑIA MINERA S.A.C. con RUC 20508440643, con una MULTA equivalente a dieciocho coma doce (18,12) UIT, por la infracción calificada como muy grave en materia de agua, por efectuar vertimiento de aguas residuales sin autorización de la Autoridad Nacional del Agua en la quebrada Fortuna, proveniente de actividad minera.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- DISPONER que el depósito de la multa impuesta sea pagada mediante depósito en las agencias del Banco de la Nación en la Cuenta Corriente N° 0000-877174 de la Autoridad Nacional del Agua (concepto multas por infracción) en el plazo de quince (15) días hábiles de notificado la presente resolución, bajo apercibimiento de iniciarse ejecución coactiva en caso de incumplimiento, debiendo alcanzar una copia del Boucher de depósito a la Administración Local de Agua Tahuamanu-Madre de Dios dentro del tercer día de efectuado el mismo.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- DISPONER como Medida Complementaria, que la NICONSTA COMPAÑIA MINERA S.A.C. con RUC 20508440643, representada por su gerente general, la Sra. Constantina Carita López identificada con DNI N° 04808544, realice el cese inmediato del vertimiento de aguas residuales hacia la quebrada Fortuna y realice los trámites necesarios para obtener la autorización de vertimiento de aguas residuales tratadas, otorgándole un plazo de hasta de seis (6) meses, computados a partir del día siguiente de la notificación de la resolución de sanción.</t>
   </si>
   <si>
     <t>1</t>
+  </si>
+  <si>
+    <t>64-RD-0250-2026-02.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0250-2026-02.pdf</t>
+  </si>
+  <si>
+    <t>64</t>
+  </si>
+  <si>
+    <t>ALA Tambopata - Inambari</t>
+  </si>
+  <si>
+    <t>0250-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>250</t>
+  </si>
+  <si>
+    <t>07/09/2026</t>
+  </si>
+  <si>
+    <t>RD N° 0250-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- DECLARAR el ABANDONO del procedimiento administrativo iniciado por la MUNICIPALIDAD DISTRITAL DE COASA con RUC N° 20159410499, sobre la solicitud de Autorización de Ejecución de Obras en Fuentes Naturales de Agua para el proyecto denominado “Mejoramiento de los servicios de protección en riberas de rio vulnerables ante el peligro en el rio Coasa del barrio Las Cantutas, distrito de Coasa de la provincia de Carabaya del departamento de Puno”, por los fundamentos expuestos en la parte considerativa de la presente resolución.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- DISPONER el ARCHIVAMIENTO DEFINITIVO del expediente administrativo una vez vencido los plazos recursivos.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- NOTIFICAR la presente resolución a la Municipalidad Distrital de Coasa a su correo electrónico señalado; poner de conocimiento a la Administración Local de Agua Tambopata-Inambari; y disponer su publicación en el portal web institucional de la Autoridad Nacional del Agua: www.ana.gob.pe.</t>
+  </si>
+  <si>
+    <t>59-RD-0251-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\59-RD-0251-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>0251-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>251</t>
+  </si>
+  <si>
+    <t>RD N° 0251-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- DECLARAR el ABANDONO del procedimiento administrativo iniciado por la MUNICIPALIDAD DISTRITAL DE KOSÑIPATA con RUC N° 20159309933, sobre la solicitud de delimitación de la faja marginal del riachuelo Aguas Santas, ubicado en el distrito de Kosñipata, provincia de Paucartambo, departamento de Cusco, por los fundamentos expuestos en la parte considerativa de la presente resolución.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- NOTIFICAR la presente resolución a la Municipalidad Distrital de Kosñipata a su correo electrónico señalado; poner de conocimiento a la Administración Local de Agua Tahuamanu-Madre de Dios; y disponer su publicación en el portal web institucional de la Autoridad Nacional del Agua: www.ana.gob.pe.</t>
+  </si>
+  <si>
+    <t>64-RD-0252-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0252-2026-03.pdf</t>
+  </si>
+  <si>
+    <t>0252-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>252</t>
+  </si>
+  <si>
+    <t>RD N° 0252-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- DECLARAR INEFICAZ Y DEJAR SIN EFECTO la Resolución Directoral Nº 0197-2026-ANA-AAA.MDD emitida el 21.07.2026, al no haberse perfeccionado su notificación legal y carecer de eficacia jurídica frente a la administrada conforme a los fundamentos expuestos en la parte considerativa de la presente resolución.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 2.- ACEPTAR el desistimiento al trámite de autorización de ejecución de obras mínimas en fuentes naturales de agua para el proyecto denominado “Ejecución de obras mínimas, protección con material propio y de préstamo, Km 186+182 LD IZQ”, ubicado en el distrito de Macusani, provincia de Carabaya, departamento de Puno, presentado en fecha 27.05.2026 por la empresa INTERSUR CONCESIONES S.A.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- DECLARAR concluido el presente procedimiento administrativo, disponiendo el archivamiento definitivo.</t>
+  </si>
+  <si>
+    <t>64-RD-0253-2026-02.pdf</t>
+  </si>
+  <si>
+    <t>D:\Datos\OneDrive - Autoridad Nacional del Agua\MDD 2026\AAA\SubirPortal\pdfs\nuevos\64-RD-0253-2026-02.pdf</t>
+  </si>
+  <si>
+    <t>0253-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>253</t>
+  </si>
+  <si>
+    <t>RD N° 0253-2026-ANA-AAA.MDD</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 1.- DECLARAR el ABANDONO del procedimiento administrativo iniciado por la MUNICIPALIDAD DISTRITAL DE CORANI con RUC N° 20205221353, sobre la solicitud de aprobación del estudio de delimitación de faja marginal del rio Izibilla - Margen Izquierdo, ubicada en el distrito de Corani, provincia de Carabaya, departamento de Puno, por los fundamentos expuestos en la parte considerativa de la presente resolución.</t>
+  </si>
+  <si>
+    <t>ARTÍCULO 3.- NOTIFICAR la presente resolución a la Municipalidad Distrital de Corani a su correo electrónico señalado; poner de conocimiento a la Administración Local de Agua Tambopata-Inambari; y disponer su publicación en el portal web institucional de la Autoridad Nacional del Agua: www.ana.gob.pe.</t>
+  </si>
+  <si>
+    <t>2</t>
   </si>
 </sst>
 </file>
@@ -168,12 +278,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -194,8 +307,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ResolucionesPendientes" displayName="ResolucionesPendientes" ref="A1:R2">
-  <autoFilter ref="A1:R2" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ResolucionesPendientes" displayName="ResolucionesPendientes" ref="A1:R6">
+  <autoFilter ref="A1:R6" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="archivo_pdf"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ruta_pdf"/>
@@ -505,8 +618,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:R6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="82" customWidth="1"/>
@@ -524,7 +637,7 @@
     <col min="18" max="18" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -580,7 +693,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" ht="87" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
@@ -608,32 +721,256 @@
       <c r="I2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J2" s="2">
-        <v>2026</v>
+      <c r="J2" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="K2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M2" s="2" t="s">
+      <c r="K3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="N2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>33</v>
+      <c r="M3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q5" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q6" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="R6" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>